<commit_message>
SCRUM-18:Test script + bugreport + kết quả kiểm thử API
</commit_message>
<xml_diff>
--- a/Docs/Test-Report/Bug_Report.xlsx
+++ b/Docs/Test-Report/Bug_Report.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\KiemChungPhanMem\Docs\Test-Report\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C51A0B6A-F0D6-42FB-AC8E-5A2F92EE716F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,10 +24,97 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
+  <si>
+    <t>Bug ID</t>
+  </si>
+  <si>
+    <t>Module</t>
+  </si>
+  <si>
+    <t>API Endpoint</t>
+  </si>
+  <si>
+    <t>Title (Tiêu đề Bug)</t>
+  </si>
+  <si>
+    <t>Severity (Mức độ)</t>
+  </si>
+  <si>
+    <t>Priority (Ưu tiên)</t>
+  </si>
+  <si>
+    <t>Expected Result (Kỳ vọng)</t>
+  </si>
+  <si>
+    <t>Actual Result (Thực tế)</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>BUG_API_002</t>
+  </si>
+  <si>
+    <t>Product</t>
+  </si>
+  <si>
+    <t>POST /api/seller/product/new</t>
+  </si>
+  <si>
+    <t>[API] Lỗi 500 do lỗi Serialize JSON (Jackson) khi bắt lỗi Validate dữ liệu thêm mới Sản phẩm</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Open</t>
+  </si>
+  <si>
+    <t>BUG_API_003</t>
+  </si>
+  <si>
+    <t>Order</t>
+  </si>
+  <si>
+    <t>[API] Lỗi 500 và sai chính tả ("is not exit!") khi thao tác với ID Đơn hàng không tồn tại</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Trả về 400 Bad Request kèm thông báo lỗi Validate cụ thể cho các field nhập sai.</t>
+  </si>
+  <si>
+    <t>Trả về 500 Internal Server Error kèm lỗi No serializer found for class... DefaultMessageCodesResolver.</t>
+  </si>
+  <si>
+    <t>Trả về 404 Not Found (hoặc 400) kèm câu thông báo chuẩn: "Order does not exist" hoặc "Order not found".</t>
+  </si>
+  <si>
+    <t>Trả về 500 Internal Server Error kèm câu thông báo sai chính tả: "OrderMain is not exit!".</t>
+  </si>
+  <si>
+    <t>GET /api/order/{id} 
+PATCH /api/order/cancel/{id} 
+PATCH /api/order/finish/{id}</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -37,7 +130,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +138,39 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +450,108 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13.109375" customWidth="1"/>
+    <col min="2" max="2" width="8.88671875" customWidth="1"/>
+    <col min="3" max="3" width="26.77734375" customWidth="1"/>
+    <col min="4" max="4" width="17.6640625" customWidth="1"/>
+    <col min="7" max="7" width="23" customWidth="1"/>
+    <col min="8" max="8" width="22.21875" customWidth="1"/>
+    <col min="9" max="9" width="8.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="72" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>